<commit_message>
NODELibrary.Timber.maple started, still buggy
</commit_message>
<xml_diff>
--- a/NODELibrary/Data/Materialdata.xlsx
+++ b/NODELibrary/Data/Materialdata.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\NODEMaple\NODELibrary\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56B9C34-7C75-40C7-AB7F-6D4D4C969952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{107753C5-EAA1-4006-9436-FABDD1C4FC02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="18240" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LESMEG" sheetId="5" r:id="rId1"/>
     <sheet name="concrete" sheetId="4" r:id="rId2"/>
     <sheet name="steel" sheetId="6" r:id="rId3"/>
-    <sheet name="tre" sheetId="3" r:id="rId4"/>
+    <sheet name="timber" sheetId="3" r:id="rId4"/>
     <sheet name="limtre" sheetId="1" r:id="rId5"/>
     <sheet name="softwood" sheetId="2" r:id="rId6"/>
     <sheet name="softwood tension tests" sheetId="7" r:id="rId7"/>

</xml_diff>